<commit_message>
chore: scrape results 2026-10-12
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -511,7 +511,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Genetic Panel Scraper — Summary  |  2026-10-05</t>
+          <t>Genetic Panel Scraper — Summary  |  2026-10-12</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       <c r="D6" s="5" t="inlineStr"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -977,7 +977,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1005,7 +1005,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1257,7 +1257,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1397,7 +1397,7 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1569,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1877,7 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2073,7 @@
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2213,7 +2213,7 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2493,7 +2493,7 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2549,7 +2549,7 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2605,7 +2605,7 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2633,7 @@
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2717,7 +2717,7 @@
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="H79" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="H83" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="H85" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3117,7 +3117,7 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="H89" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3173,7 +3173,7 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="H91" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="H93" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3289,7 +3289,7 @@
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="H95" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3373,7 +3373,7 @@
       </c>
       <c r="H97" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="H99" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3461,7 +3461,7 @@
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="H101" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="H103" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3573,7 +3573,7 @@
       </c>
       <c r="H104" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="H105" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3633,7 +3633,7 @@
       </c>
       <c r="H106" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="H107" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3689,7 +3689,7 @@
       </c>
       <c r="H108" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="H109" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3745,7 @@
       </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3777,7 +3777,7 @@
       </c>
       <c r="H111" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3805,7 +3805,7 @@
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="H113" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3889,7 +3889,7 @@
       </c>
       <c r="H115" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3917,7 +3917,7 @@
       </c>
       <c r="H116" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3945,7 +3945,7 @@
       </c>
       <c r="H117" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="H119" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4029,7 +4029,7 @@
       </c>
       <c r="H120" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="H121" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="H122" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4113,7 +4113,7 @@
       </c>
       <c r="H123" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4141,7 @@
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4169,7 +4169,7 @@
       </c>
       <c r="H125" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="H126" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4225,7 +4225,7 @@
       </c>
       <c r="H127" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4253,7 +4253,7 @@
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="H129" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4309,7 +4309,7 @@
       </c>
       <c r="H130" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4337,7 +4337,7 @@
       </c>
       <c r="H131" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4365,7 +4365,7 @@
       </c>
       <c r="H132" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4393,7 +4393,7 @@
       </c>
       <c r="H133" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4421,7 +4421,7 @@
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4449,7 +4449,7 @@
       </c>
       <c r="H135" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4477,7 +4477,7 @@
       </c>
       <c r="H136" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="H137" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4533,7 +4533,7 @@
       </c>
       <c r="H138" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4561,7 @@
       </c>
       <c r="H139" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4589,7 +4589,7 @@
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4617,7 +4617,7 @@
       </c>
       <c r="H141" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4645,7 +4645,7 @@
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="H143" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4705,7 +4705,7 @@
       </c>
       <c r="H144" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4733,7 +4733,7 @@
       </c>
       <c r="H145" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4761,7 +4761,7 @@
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4789,7 +4789,7 @@
       </c>
       <c r="H147" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4817,7 +4817,7 @@
       </c>
       <c r="H148" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="H149" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4873,7 +4873,7 @@
       </c>
       <c r="H150" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="H151" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4929,7 +4929,7 @@
       </c>
       <c r="H152" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="H153" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -4985,7 +4985,7 @@
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5013,7 +5013,7 @@
       </c>
       <c r="H155" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5041,7 +5041,7 @@
       </c>
       <c r="H156" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5069,7 +5069,7 @@
       </c>
       <c r="H157" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5097,7 +5097,7 @@
       </c>
       <c r="H158" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5125,7 +5125,7 @@
       </c>
       <c r="H159" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="H160" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5181,7 +5181,7 @@
       </c>
       <c r="H161" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5213,7 +5213,7 @@
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5241,7 +5241,7 @@
       </c>
       <c r="H163" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5269,7 +5269,7 @@
       </c>
       <c r="H164" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5297,7 +5297,7 @@
       </c>
       <c r="H165" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5329,7 +5329,7 @@
       </c>
       <c r="H166" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5357,7 +5357,7 @@
       </c>
       <c r="H167" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5413,7 +5413,7 @@
       </c>
       <c r="H169" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5441,7 +5441,7 @@
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="H171" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5497,7 +5497,7 @@
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5525,7 +5525,7 @@
       </c>
       <c r="H173" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="H174" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5581,7 +5581,7 @@
       </c>
       <c r="H175" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5613,7 +5613,7 @@
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5641,7 +5641,7 @@
       </c>
       <c r="H177" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5673,7 +5673,7 @@
       </c>
       <c r="H178" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5701,7 @@
       </c>
       <c r="H179" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5729,7 +5729,7 @@
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5757,7 +5757,7 @@
       </c>
       <c r="H181" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5785,7 +5785,7 @@
       </c>
       <c r="H182" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5813,7 +5813,7 @@
       </c>
       <c r="H183" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5845,7 +5845,7 @@
       </c>
       <c r="H184" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5873,7 +5873,7 @@
       </c>
       <c r="H185" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5901,7 +5901,7 @@
       </c>
       <c r="H186" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5929,7 +5929,7 @@
       </c>
       <c r="H187" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5957,7 +5957,7 @@
       </c>
       <c r="H188" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5989,7 +5989,7 @@
       </c>
       <c r="H189" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6017,7 +6017,7 @@
       </c>
       <c r="H190" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6045,7 +6045,7 @@
       </c>
       <c r="H191" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6073,7 +6073,7 @@
       </c>
       <c r="H192" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6101,7 +6101,7 @@
       </c>
       <c r="H193" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6129,7 +6129,7 @@
       </c>
       <c r="H194" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6157,7 +6157,7 @@
       </c>
       <c r="H195" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6189,7 +6189,7 @@
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6217,7 +6217,7 @@
       </c>
       <c r="H197" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6245,7 +6245,7 @@
       </c>
       <c r="H198" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6273,7 +6273,7 @@
       </c>
       <c r="H199" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6301,7 +6301,7 @@
       </c>
       <c r="H200" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="H201" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6357,7 @@
       </c>
       <c r="H202" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6385,7 +6385,7 @@
       </c>
       <c r="H203" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6413,7 +6413,7 @@
       </c>
       <c r="H204" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
       </c>
       <c r="H205" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6473,7 +6473,7 @@
       </c>
       <c r="H206" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6501,7 +6501,7 @@
       </c>
       <c r="H207" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6529,7 +6529,7 @@
       </c>
       <c r="H208" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6557,7 +6557,7 @@
       </c>
       <c r="H209" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6585,7 +6585,7 @@
       </c>
       <c r="H210" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6613,7 +6613,7 @@
       </c>
       <c r="H211" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6641,7 +6641,7 @@
       </c>
       <c r="H212" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6669,7 +6669,7 @@
       </c>
       <c r="H213" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6697,7 +6697,7 @@
       </c>
       <c r="H214" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6725,7 +6725,7 @@
       </c>
       <c r="H215" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6753,7 +6753,7 @@
       </c>
       <c r="H216" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6781,7 +6781,7 @@
       </c>
       <c r="H217" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6809,7 +6809,7 @@
       </c>
       <c r="H218" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6837,7 +6837,7 @@
       </c>
       <c r="H219" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6865,7 +6865,7 @@
       </c>
       <c r="H220" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6893,7 +6893,7 @@
       </c>
       <c r="H221" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="H222" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6949,7 +6949,7 @@
       </c>
       <c r="H223" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="H224" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7009,7 +7009,7 @@
       </c>
       <c r="H225" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7037,7 +7037,7 @@
       </c>
       <c r="H226" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="H227" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7093,7 +7093,7 @@
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7121,7 +7121,7 @@
       </c>
       <c r="H229" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="H230" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7177,7 +7177,7 @@
       </c>
       <c r="H231" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7205,7 +7205,7 @@
       </c>
       <c r="H232" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7233,7 +7233,7 @@
       </c>
       <c r="H233" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7261,7 +7261,7 @@
       </c>
       <c r="H234" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7289,7 +7289,7 @@
       </c>
       <c r="H235" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7317,7 +7317,7 @@
       </c>
       <c r="H236" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7345,7 +7345,7 @@
       </c>
       <c r="H237" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7373,7 +7373,7 @@
       </c>
       <c r="H238" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7401,7 +7401,7 @@
       </c>
       <c r="H239" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7429,7 +7429,7 @@
       </c>
       <c r="H240" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7457,7 +7457,7 @@
       </c>
       <c r="H241" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7485,7 +7485,7 @@
       </c>
       <c r="H242" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7513,7 +7513,7 @@
       </c>
       <c r="H243" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7541,7 +7541,7 @@
       </c>
       <c r="H244" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7569,7 +7569,7 @@
       </c>
       <c r="H245" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7597,7 +7597,7 @@
       </c>
       <c r="H246" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7625,7 +7625,7 @@
       </c>
       <c r="H247" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7653,7 +7653,7 @@
       </c>
       <c r="H248" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7681,7 +7681,7 @@
       </c>
       <c r="H249" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7709,7 +7709,7 @@
       </c>
       <c r="H250" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7737,7 +7737,7 @@
       </c>
       <c r="H251" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7765,7 +7765,7 @@
       </c>
       <c r="H252" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7793,7 +7793,7 @@
       </c>
       <c r="H253" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7825,7 +7825,7 @@
       </c>
       <c r="H254" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7857,7 +7857,7 @@
       </c>
       <c r="H255" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7889,7 +7889,7 @@
       </c>
       <c r="H256" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7921,7 +7921,7 @@
       </c>
       <c r="H257" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7953,7 +7953,7 @@
       </c>
       <c r="H258" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7985,7 +7985,7 @@
       </c>
       <c r="H259" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8017,7 +8017,7 @@
       </c>
       <c r="H260" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8049,7 +8049,7 @@
       </c>
       <c r="H261" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="H262" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8113,7 +8113,7 @@
       </c>
       <c r="H263" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8145,7 +8145,7 @@
       </c>
       <c r="H264" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8177,7 +8177,7 @@
       </c>
       <c r="H265" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8209,7 +8209,7 @@
       </c>
       <c r="H266" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8241,7 +8241,7 @@
       </c>
       <c r="H267" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8273,7 +8273,7 @@
       </c>
       <c r="H268" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8305,7 +8305,7 @@
       </c>
       <c r="H269" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8337,7 +8337,7 @@
       </c>
       <c r="H270" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8369,7 +8369,7 @@
       </c>
       <c r="H271" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8401,7 +8401,7 @@
       </c>
       <c r="H272" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8433,7 +8433,7 @@
       </c>
       <c r="H273" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8465,7 +8465,7 @@
       </c>
       <c r="H274" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8497,7 +8497,7 @@
       </c>
       <c r="H275" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8529,7 +8529,7 @@
       </c>
       <c r="H276" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8561,7 +8561,7 @@
       </c>
       <c r="H277" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8593,7 +8593,7 @@
       </c>
       <c r="H278" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8625,7 +8625,7 @@
       </c>
       <c r="H279" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8657,7 +8657,7 @@
       </c>
       <c r="H280" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8689,7 +8689,7 @@
       </c>
       <c r="H281" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8721,7 +8721,7 @@
       </c>
       <c r="H282" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8753,7 +8753,7 @@
       </c>
       <c r="H283" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8785,7 +8785,7 @@
       </c>
       <c r="H284" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8817,7 +8817,7 @@
       </c>
       <c r="H285" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8849,7 +8849,7 @@
       </c>
       <c r="H286" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8881,7 +8881,7 @@
       </c>
       <c r="H287" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8913,7 +8913,7 @@
       </c>
       <c r="H288" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8945,7 +8945,7 @@
       </c>
       <c r="H289" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -8977,7 +8977,7 @@
       </c>
       <c r="H290" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -9009,7 +9009,7 @@
       </c>
       <c r="H291" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -9041,7 +9041,7 @@
       </c>
       <c r="H292" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -9073,7 +9073,7 @@
       </c>
       <c r="H293" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -9105,7 +9105,7 @@
       </c>
       <c r="H294" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -9137,7 +9137,7 @@
       </c>
       <c r="H295" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -9169,7 +9169,7 @@
       </c>
       <c r="H296" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -9201,7 +9201,7 @@
       </c>
       <c r="H297" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -9233,7 +9233,7 @@
       </c>
       <c r="H298" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -9265,7 +9265,7 @@
       </c>
       <c r="H299" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -9297,7 +9297,7 @@
       </c>
       <c r="H300" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: scrape results 2026-10-19
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -511,7 +511,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Genetic Panel Scraper — Summary  |  2026-10-12</t>
+          <t>Genetic Panel Scraper — Summary  |  2026-10-19</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>0</v>
@@ -581,7 +581,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>0</v>
@@ -600,7 +600,7 @@
       <c r="D6" s="5" t="inlineStr"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H300"/>
+  <dimension ref="A1:H299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -697,7 +697,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -977,7 +977,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1005,7 +1005,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1257,7 +1257,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1397,7 +1397,7 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1569,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1877,7 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2073,7 @@
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2213,7 +2213,7 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2493,7 +2493,7 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2549,7 +2549,7 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2605,7 +2605,7 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2633,7 @@
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2717,7 +2717,7 @@
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="H79" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="H83" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="H85" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3117,7 +3117,7 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="H89" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3173,7 +3173,7 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="H91" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="H93" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3289,7 +3289,7 @@
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="H95" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3373,7 +3373,7 @@
       </c>
       <c r="H97" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="H99" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3461,7 +3461,7 @@
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="H101" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="H103" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3573,7 +3573,7 @@
       </c>
       <c r="H104" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="H105" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3633,7 +3633,7 @@
       </c>
       <c r="H106" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="H107" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3689,7 +3689,7 @@
       </c>
       <c r="H108" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="H109" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3745,7 @@
       </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3777,7 +3777,7 @@
       </c>
       <c r="H111" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3805,7 +3805,7 @@
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="H113" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3889,7 +3889,7 @@
       </c>
       <c r="H115" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3917,7 +3917,7 @@
       </c>
       <c r="H116" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3945,7 +3945,7 @@
       </c>
       <c r="H117" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="H119" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4029,7 +4029,7 @@
       </c>
       <c r="H120" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="H121" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="H122" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4113,7 +4113,7 @@
       </c>
       <c r="H123" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4141,7 @@
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4169,7 +4169,7 @@
       </c>
       <c r="H125" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="H126" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4225,7 +4225,7 @@
       </c>
       <c r="H127" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4253,7 +4253,7 @@
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="H129" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4309,7 +4309,7 @@
       </c>
       <c r="H130" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4337,7 +4337,7 @@
       </c>
       <c r="H131" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4365,7 +4365,7 @@
       </c>
       <c r="H132" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4393,7 +4393,7 @@
       </c>
       <c r="H133" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4421,7 +4421,7 @@
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4449,7 +4449,7 @@
       </c>
       <c r="H135" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4477,7 +4477,7 @@
       </c>
       <c r="H136" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="H137" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4533,7 +4533,7 @@
       </c>
       <c r="H138" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4561,7 @@
       </c>
       <c r="H139" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4589,7 +4589,7 @@
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4617,7 +4617,7 @@
       </c>
       <c r="H141" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4645,7 +4645,7 @@
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="H143" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4705,7 +4705,7 @@
       </c>
       <c r="H144" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4733,7 +4733,7 @@
       </c>
       <c r="H145" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4761,7 +4761,7 @@
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4789,7 +4789,7 @@
       </c>
       <c r="H147" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4817,7 +4817,7 @@
       </c>
       <c r="H148" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="H149" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4873,7 +4873,7 @@
       </c>
       <c r="H150" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="H151" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4929,7 +4929,7 @@
       </c>
       <c r="H152" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="H153" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4985,7 +4985,7 @@
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5013,7 +5013,7 @@
       </c>
       <c r="H155" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5041,7 +5041,7 @@
       </c>
       <c r="H156" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5069,7 +5069,7 @@
       </c>
       <c r="H157" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5097,7 +5097,7 @@
       </c>
       <c r="H158" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5125,7 +5125,7 @@
       </c>
       <c r="H159" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="H160" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5181,7 +5181,7 @@
       </c>
       <c r="H161" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5213,7 +5213,7 @@
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5241,7 +5241,7 @@
       </c>
       <c r="H163" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5269,7 +5269,7 @@
       </c>
       <c r="H164" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5297,7 +5297,7 @@
       </c>
       <c r="H165" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5329,7 +5329,7 @@
       </c>
       <c r="H166" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5357,7 +5357,7 @@
       </c>
       <c r="H167" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5413,7 +5413,7 @@
       </c>
       <c r="H169" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5441,7 +5441,7 @@
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="H171" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5497,7 +5497,7 @@
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5525,7 +5525,7 @@
       </c>
       <c r="H173" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="H174" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5581,7 +5581,7 @@
       </c>
       <c r="H175" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5613,7 +5613,7 @@
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5641,7 +5641,7 @@
       </c>
       <c r="H177" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5673,7 +5673,7 @@
       </c>
       <c r="H178" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5701,7 @@
       </c>
       <c r="H179" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5729,7 +5729,7 @@
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5757,7 +5757,7 @@
       </c>
       <c r="H181" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5785,7 +5785,7 @@
       </c>
       <c r="H182" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5813,7 +5813,7 @@
       </c>
       <c r="H183" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5845,7 +5845,7 @@
       </c>
       <c r="H184" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5873,7 +5873,7 @@
       </c>
       <c r="H185" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5901,7 +5901,7 @@
       </c>
       <c r="H186" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5929,7 +5929,7 @@
       </c>
       <c r="H187" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5957,7 +5957,7 @@
       </c>
       <c r="H188" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5989,7 +5989,7 @@
       </c>
       <c r="H189" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6017,7 +6017,7 @@
       </c>
       <c r="H190" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6045,7 +6045,7 @@
       </c>
       <c r="H191" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6073,7 +6073,7 @@
       </c>
       <c r="H192" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6101,7 +6101,7 @@
       </c>
       <c r="H193" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6129,7 +6129,7 @@
       </c>
       <c r="H194" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6157,7 +6157,7 @@
       </c>
       <c r="H195" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6189,7 +6189,7 @@
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6217,7 +6217,7 @@
       </c>
       <c r="H197" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6245,7 +6245,7 @@
       </c>
       <c r="H198" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6273,7 +6273,7 @@
       </c>
       <c r="H199" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6301,7 +6301,7 @@
       </c>
       <c r="H200" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="H201" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6357,7 @@
       </c>
       <c r="H202" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6385,7 +6385,7 @@
       </c>
       <c r="H203" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6413,7 +6413,7 @@
       </c>
       <c r="H204" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
       </c>
       <c r="H205" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6473,7 +6473,7 @@
       </c>
       <c r="H206" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6501,7 +6501,7 @@
       </c>
       <c r="H207" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6529,7 +6529,7 @@
       </c>
       <c r="H208" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6557,7 +6557,7 @@
       </c>
       <c r="H209" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6585,7 +6585,7 @@
       </c>
       <c r="H210" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6613,7 +6613,7 @@
       </c>
       <c r="H211" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6641,7 +6641,7 @@
       </c>
       <c r="H212" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6669,7 +6669,7 @@
       </c>
       <c r="H213" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6697,7 +6697,7 @@
       </c>
       <c r="H214" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6725,7 +6725,7 @@
       </c>
       <c r="H215" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6753,7 +6753,7 @@
       </c>
       <c r="H216" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6781,7 +6781,7 @@
       </c>
       <c r="H217" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6809,7 +6809,7 @@
       </c>
       <c r="H218" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6837,7 +6837,7 @@
       </c>
       <c r="H219" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6865,7 +6865,7 @@
       </c>
       <c r="H220" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6893,7 +6893,7 @@
       </c>
       <c r="H221" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="H222" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6949,7 +6949,7 @@
       </c>
       <c r="H223" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="H224" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7009,7 +7009,7 @@
       </c>
       <c r="H225" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7037,7 +7037,7 @@
       </c>
       <c r="H226" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="H227" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7093,7 +7093,7 @@
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7121,7 +7121,7 @@
       </c>
       <c r="H229" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="H230" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7177,7 +7177,7 @@
       </c>
       <c r="H231" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7205,7 +7205,7 @@
       </c>
       <c r="H232" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7233,7 +7233,7 @@
       </c>
       <c r="H233" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7261,7 +7261,7 @@
       </c>
       <c r="H234" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7289,7 +7289,7 @@
       </c>
       <c r="H235" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7317,7 +7317,7 @@
       </c>
       <c r="H236" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7345,7 +7345,7 @@
       </c>
       <c r="H237" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7373,7 +7373,7 @@
       </c>
       <c r="H238" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7401,7 +7401,7 @@
       </c>
       <c r="H239" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7429,7 +7429,7 @@
       </c>
       <c r="H240" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7457,7 +7457,7 @@
       </c>
       <c r="H241" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7485,7 +7485,7 @@
       </c>
       <c r="H242" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7513,7 +7513,7 @@
       </c>
       <c r="H243" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7541,7 +7541,7 @@
       </c>
       <c r="H244" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7569,7 +7569,7 @@
       </c>
       <c r="H245" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7597,7 +7597,7 @@
       </c>
       <c r="H246" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7625,7 +7625,7 @@
       </c>
       <c r="H247" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7653,7 +7653,7 @@
       </c>
       <c r="H248" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7681,7 +7681,7 @@
       </c>
       <c r="H249" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7709,7 +7709,7 @@
       </c>
       <c r="H250" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7737,7 +7737,7 @@
       </c>
       <c r="H251" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7765,7 +7765,7 @@
       </c>
       <c r="H252" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7793,7 +7793,7 @@
       </c>
       <c r="H253" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7825,7 +7825,7 @@
       </c>
       <c r="H254" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7857,7 +7857,7 @@
       </c>
       <c r="H255" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7889,7 +7889,7 @@
       </c>
       <c r="H256" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7921,7 +7921,7 @@
       </c>
       <c r="H257" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7953,7 +7953,7 @@
       </c>
       <c r="H258" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7985,7 +7985,7 @@
       </c>
       <c r="H259" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8017,7 +8017,7 @@
       </c>
       <c r="H260" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8049,7 +8049,7 @@
       </c>
       <c r="H261" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="H262" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8113,7 +8113,7 @@
       </c>
       <c r="H263" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8145,7 +8145,7 @@
       </c>
       <c r="H264" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8177,7 +8177,7 @@
       </c>
       <c r="H265" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8209,7 +8209,7 @@
       </c>
       <c r="H266" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8241,7 +8241,7 @@
       </c>
       <c r="H267" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8273,7 +8273,7 @@
       </c>
       <c r="H268" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8305,7 +8305,7 @@
       </c>
       <c r="H269" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8337,7 +8337,7 @@
       </c>
       <c r="H270" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8369,7 +8369,7 @@
       </c>
       <c r="H271" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8401,7 +8401,7 @@
       </c>
       <c r="H272" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8433,7 +8433,7 @@
       </c>
       <c r="H273" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8465,7 +8465,7 @@
       </c>
       <c r="H274" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8497,7 +8497,7 @@
       </c>
       <c r="H275" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8529,7 +8529,7 @@
       </c>
       <c r="H276" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8561,7 +8561,7 @@
       </c>
       <c r="H277" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8593,7 +8593,7 @@
       </c>
       <c r="H278" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8605,7 +8605,7 @@
       </c>
       <c r="B279" s="7" t="inlineStr">
         <is>
-          <t>Pharma Services</t>
+          <t>Pricing and Billing Information</t>
         </is>
       </c>
       <c r="C279" s="4" t="inlineStr"/>
@@ -8620,12 +8620,12 @@
       <c r="F279" s="7" t="inlineStr"/>
       <c r="G279" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/renasight-genetic-testing/pharma-research/</t>
+          <t>https://www.natera.com/oncology/billing/</t>
         </is>
       </c>
       <c r="H279" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8652,12 +8652,12 @@
       <c r="F280" s="6" t="inlineStr"/>
       <c r="G280" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/oncology/billing/</t>
+          <t>https://www.natera.com/organ-health/organ-health-pricing-billing/</t>
         </is>
       </c>
       <c r="H280" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8684,12 +8684,12 @@
       <c r="F281" s="7" t="inlineStr"/>
       <c r="G281" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/organ-health-pricing-billing/</t>
+          <t>https://www.natera.com/womens-health/pricing-billing/</t>
         </is>
       </c>
       <c r="H281" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8701,7 +8701,7 @@
       </c>
       <c r="B282" s="6" t="inlineStr">
         <is>
-          <t>Pricing and Billing Information</t>
+          <t>Prospera™ Heart–Transplant Assessment</t>
         </is>
       </c>
       <c r="C282" s="3" t="inlineStr"/>
@@ -8716,12 +8716,12 @@
       <c r="F282" s="6" t="inlineStr"/>
       <c r="G282" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/womens-health/pricing-billing/</t>
+          <t>https://www.natera.com/organ-health/prospera-heart-transplantation-assessment/</t>
         </is>
       </c>
       <c r="H282" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8733,7 +8733,7 @@
       </c>
       <c r="B283" s="7" t="inlineStr">
         <is>
-          <t>Prospera™ Heart–Transplant Assessment</t>
+          <t>Prospera™ Kidney–Transplant Assessment</t>
         </is>
       </c>
       <c r="C283" s="4" t="inlineStr"/>
@@ -8748,12 +8748,12 @@
       <c r="F283" s="7" t="inlineStr"/>
       <c r="G283" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-heart-transplantation-assessment/</t>
+          <t>https://www.natera.com/organ-health/prospera-organ-transplantation-assessment/</t>
         </is>
       </c>
       <c r="H283" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8765,7 +8765,7 @@
       </c>
       <c r="B284" s="6" t="inlineStr">
         <is>
-          <t>Prospera™ Kidney–Transplant Assessment</t>
+          <t>Prospera™ Liver–Transplant Assessment</t>
         </is>
       </c>
       <c r="C284" s="3" t="inlineStr"/>
@@ -8780,12 +8780,12 @@
       <c r="F284" s="6" t="inlineStr"/>
       <c r="G284" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-organ-transplantation-assessment/</t>
+          <t>https://www.natera.com/organ-health/prospera-liver-transplantation-assessment/</t>
         </is>
       </c>
       <c r="H284" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8797,7 +8797,7 @@
       </c>
       <c r="B285" s="7" t="inlineStr">
         <is>
-          <t>Prospera™ Liver–Transplant Assessment</t>
+          <t>Prospera™ Lung–Transplant Assessment</t>
         </is>
       </c>
       <c r="C285" s="4" t="inlineStr"/>
@@ -8812,12 +8812,12 @@
       <c r="F285" s="7" t="inlineStr"/>
       <c r="G285" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-liver-transplantation-assessment/</t>
+          <t>https://www.natera.com/organ-health/prospera-lung-transplantation-assessment/</t>
         </is>
       </c>
       <c r="H285" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8829,7 +8829,7 @@
       </c>
       <c r="B286" s="6" t="inlineStr">
         <is>
-          <t>Prospera™ Lung–Transplant Assessment</t>
+          <t>Prospera™ for Heart Patients</t>
         </is>
       </c>
       <c r="C286" s="3" t="inlineStr"/>
@@ -8844,12 +8844,12 @@
       <c r="F286" s="6" t="inlineStr"/>
       <c r="G286" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-lung-transplantation-assessment/</t>
+          <t>https://www.natera.com/organ-health/prospera-heart-transplantation-assessment/patients/</t>
         </is>
       </c>
       <c r="H286" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8861,7 +8861,7 @@
       </c>
       <c r="B287" s="7" t="inlineStr">
         <is>
-          <t>Prospera™ for Heart Patients</t>
+          <t>Prospera™ for Kidney Clinician</t>
         </is>
       </c>
       <c r="C287" s="4" t="inlineStr"/>
@@ -8876,12 +8876,12 @@
       <c r="F287" s="7" t="inlineStr"/>
       <c r="G287" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-heart-transplantation-assessment/patients/</t>
+          <t>https://www.natera.com/organ-health/prospera-organ-transplantation-assessment/clinicians/</t>
         </is>
       </c>
       <c r="H287" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8893,7 +8893,7 @@
       </c>
       <c r="B288" s="6" t="inlineStr">
         <is>
-          <t>Prospera™ for Kidney Clinician</t>
+          <t>Prospera™ for Kidney Patients</t>
         </is>
       </c>
       <c r="C288" s="3" t="inlineStr"/>
@@ -8908,12 +8908,12 @@
       <c r="F288" s="6" t="inlineStr"/>
       <c r="G288" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-organ-transplantation-assessment/clinicians/</t>
+          <t>https://www.natera.com/organ-health/prospera-organ-transplantation-assessment/patients/</t>
         </is>
       </c>
       <c r="H288" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8925,7 +8925,7 @@
       </c>
       <c r="B289" s="7" t="inlineStr">
         <is>
-          <t>Prospera™ for Kidney Patients</t>
+          <t>Prospera™ for Lung Patients</t>
         </is>
       </c>
       <c r="C289" s="4" t="inlineStr"/>
@@ -8940,12 +8940,12 @@
       <c r="F289" s="7" t="inlineStr"/>
       <c r="G289" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-organ-transplantation-assessment/patients/</t>
+          <t>https://www.natera.com/organ-health/prospera-lung-transplantation-assessment/patients/</t>
         </is>
       </c>
       <c r="H289" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8957,7 +8957,7 @@
       </c>
       <c r="B290" s="6" t="inlineStr">
         <is>
-          <t>Prospera™ for Lung Patients</t>
+          <t>Renasight™ Clinician Information</t>
         </is>
       </c>
       <c r="C290" s="3" t="inlineStr"/>
@@ -8972,12 +8972,12 @@
       <c r="F290" s="6" t="inlineStr"/>
       <c r="G290" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-lung-transplantation-assessment/patients/</t>
+          <t>https://www.natera.com/organ-health/renasight-genetic-testing/clinicians/#pg-menu-tabs</t>
         </is>
       </c>
       <c r="H290" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8989,7 +8989,7 @@
       </c>
       <c r="B291" s="7" t="inlineStr">
         <is>
-          <t>Renasight™ Clinician Information</t>
+          <t>Renasight™ Gene Conditions List</t>
         </is>
       </c>
       <c r="C291" s="4" t="inlineStr"/>
@@ -9004,12 +9004,12 @@
       <c r="F291" s="7" t="inlineStr"/>
       <c r="G291" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/renasight-genetic-testing/clinicians/#pg-menu-tabs</t>
+          <t>https://www.natera.com/organ-health/renasight-genetic-testing/gene-conditions-list/</t>
         </is>
       </c>
       <c r="H291" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -9021,7 +9021,7 @@
       </c>
       <c r="B292" s="6" t="inlineStr">
         <is>
-          <t>Renasight™ Gene Conditions List</t>
+          <t>Renasight™ Patient Information</t>
         </is>
       </c>
       <c r="C292" s="3" t="inlineStr"/>
@@ -9036,12 +9036,12 @@
       <c r="F292" s="6" t="inlineStr"/>
       <c r="G292" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/renasight-genetic-testing/gene-conditions-list/</t>
+          <t>https://www.natera.com/organ-health/renasight-genetic-testing/patients/</t>
         </is>
       </c>
       <c r="H292" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -9053,7 +9053,7 @@
       </c>
       <c r="B293" s="7" t="inlineStr">
         <is>
-          <t>Renasight™ Patient Information</t>
+          <t>Renasight™–Kidney Gene Panel</t>
         </is>
       </c>
       <c r="C293" s="4" t="inlineStr"/>
@@ -9068,12 +9068,12 @@
       <c r="F293" s="7" t="inlineStr"/>
       <c r="G293" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/renasight-genetic-testing/patients/</t>
+          <t>https://www.natera.com/organ-health/renasight-genetic-testing/</t>
         </is>
       </c>
       <c r="H293" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -9085,7 +9085,7 @@
       </c>
       <c r="B294" s="6" t="inlineStr">
         <is>
-          <t>Renasight™–Kidney Gene Panel</t>
+          <t>Signatera™ Clinician Information</t>
         </is>
       </c>
       <c r="C294" s="3" t="inlineStr"/>
@@ -9100,12 +9100,12 @@
       <c r="F294" s="6" t="inlineStr"/>
       <c r="G294" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/renasight-genetic-testing/</t>
+          <t>https://www.natera.com/oncology/signatera-advanced-cancer-detection/clinicians/</t>
         </is>
       </c>
       <c r="H294" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -9117,7 +9117,7 @@
       </c>
       <c r="B295" s="7" t="inlineStr">
         <is>
-          <t>Signatera™ Clinician Information</t>
+          <t>Signatera™ Patient Information</t>
         </is>
       </c>
       <c r="C295" s="4" t="inlineStr"/>
@@ -9132,12 +9132,12 @@
       <c r="F295" s="7" t="inlineStr"/>
       <c r="G295" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/oncology/signatera-advanced-cancer-detection/clinicians/</t>
+          <t>https://www.natera.com/oncology/signatera-advanced-cancer-detection/patients/</t>
         </is>
       </c>
       <c r="H295" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -9149,7 +9149,7 @@
       </c>
       <c r="B296" s="6" t="inlineStr">
         <is>
-          <t>Signatera™ Patient Information</t>
+          <t>Signatera™–Residual Disease Test (MRD)</t>
         </is>
       </c>
       <c r="C296" s="3" t="inlineStr"/>
@@ -9164,12 +9164,12 @@
       <c r="F296" s="6" t="inlineStr"/>
       <c r="G296" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/oncology/signatera-advanced-cancer-detection/patients/</t>
+          <t>https://www.natera.com/oncology/signatera-advanced-cancer-detection/</t>
         </is>
       </c>
       <c r="H296" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -9181,7 +9181,7 @@
       </c>
       <c r="B297" s="7" t="inlineStr">
         <is>
-          <t>Signatera™–Residual Disease Test (MRD)</t>
+          <t>Vasistera™–Limited Noninvasive Prenatal Testing (NIPT)</t>
         </is>
       </c>
       <c r="C297" s="4" t="inlineStr"/>
@@ -9196,12 +9196,12 @@
       <c r="F297" s="7" t="inlineStr"/>
       <c r="G297" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/oncology/signatera-advanced-cancer-detection/</t>
+          <t>https://www.natera.com/womens-health/vasistera/</t>
         </is>
       </c>
       <c r="H297" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -9213,7 +9213,7 @@
       </c>
       <c r="B298" s="6" t="inlineStr">
         <is>
-          <t>Vasistera™–Limited Noninvasive Prenatal Testing (NIPT)</t>
+          <t>Vistara™–Single-Gene NIPT</t>
         </is>
       </c>
       <c r="C298" s="3" t="inlineStr"/>
@@ -9228,12 +9228,12 @@
       <c r="F298" s="6" t="inlineStr"/>
       <c r="G298" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/womens-health/vasistera/</t>
+          <t>https://www.natera.com/womens-health/vistara-nipt-single-gene-test/</t>
         </is>
       </c>
       <c r="H298" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -9245,13 +9245,13 @@
       </c>
       <c r="B299" s="7" t="inlineStr">
         <is>
-          <t>Vistara™–Single-Gene NIPT</t>
+          <t>Women’s Health</t>
         </is>
       </c>
       <c r="C299" s="4" t="inlineStr"/>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>Womens Health</t>
+          <t>Organ Health</t>
         </is>
       </c>
       <c r="E299" s="4" t="n">
@@ -9260,44 +9260,12 @@
       <c r="F299" s="7" t="inlineStr"/>
       <c r="G299" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/womens-health/vistara-nipt-single-gene-test/</t>
+          <t>https://www.natera.com/womens-health/</t>
         </is>
       </c>
       <c r="H299" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="300">
-      <c r="A300" s="3" t="inlineStr">
-        <is>
-          <t>Natera</t>
-        </is>
-      </c>
-      <c r="B300" s="6" t="inlineStr">
-        <is>
-          <t>Women’s Health</t>
-        </is>
-      </c>
-      <c r="C300" s="3" t="inlineStr"/>
-      <c r="D300" s="3" t="inlineStr">
-        <is>
-          <t>Organ Health</t>
-        </is>
-      </c>
-      <c r="E300" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F300" s="6" t="inlineStr"/>
-      <c r="G300" s="6" t="inlineStr">
-        <is>
-          <t>https://www.natera.com/womens-health/</t>
-        </is>
-      </c>
-      <c r="H300" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -13970,7 +13938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -14566,7 +14534,7 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Pharma Services</t>
+          <t>Pricing and Billing Information</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr"/>
@@ -14581,7 +14549,7 @@
       <c r="E27" s="7" t="inlineStr"/>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/renasight-genetic-testing/pharma-research/</t>
+          <t>https://www.natera.com/oncology/billing/</t>
         </is>
       </c>
     </row>
@@ -14603,7 +14571,7 @@
       <c r="E28" s="6" t="inlineStr"/>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/oncology/billing/</t>
+          <t>https://www.natera.com/organ-health/organ-health-pricing-billing/</t>
         </is>
       </c>
     </row>
@@ -14625,14 +14593,14 @@
       <c r="E29" s="7" t="inlineStr"/>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/organ-health-pricing-billing/</t>
+          <t>https://www.natera.com/womens-health/pricing-billing/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Pricing and Billing Information</t>
+          <t>Prospera™ Heart–Transplant Assessment</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr"/>
@@ -14647,14 +14615,14 @@
       <c r="E30" s="6" t="inlineStr"/>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/womens-health/pricing-billing/</t>
+          <t>https://www.natera.com/organ-health/prospera-heart-transplantation-assessment/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Prospera™ Heart–Transplant Assessment</t>
+          <t>Prospera™ Kidney–Transplant Assessment</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr"/>
@@ -14669,14 +14637,14 @@
       <c r="E31" s="7" t="inlineStr"/>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-heart-transplantation-assessment/</t>
+          <t>https://www.natera.com/organ-health/prospera-organ-transplantation-assessment/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Prospera™ Kidney–Transplant Assessment</t>
+          <t>Prospera™ Liver–Transplant Assessment</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr"/>
@@ -14691,14 +14659,14 @@
       <c r="E32" s="6" t="inlineStr"/>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-organ-transplantation-assessment/</t>
+          <t>https://www.natera.com/organ-health/prospera-liver-transplantation-assessment/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Prospera™ Liver–Transplant Assessment</t>
+          <t>Prospera™ Lung–Transplant Assessment</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr"/>
@@ -14713,14 +14681,14 @@
       <c r="E33" s="7" t="inlineStr"/>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-liver-transplantation-assessment/</t>
+          <t>https://www.natera.com/organ-health/prospera-lung-transplantation-assessment/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Prospera™ Lung–Transplant Assessment</t>
+          <t>Prospera™ for Heart Patients</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr"/>
@@ -14735,14 +14703,14 @@
       <c r="E34" s="6" t="inlineStr"/>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-lung-transplantation-assessment/</t>
+          <t>https://www.natera.com/organ-health/prospera-heart-transplantation-assessment/patients/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Prospera™ for Heart Patients</t>
+          <t>Prospera™ for Kidney Clinician</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr"/>
@@ -14757,14 +14725,14 @@
       <c r="E35" s="7" t="inlineStr"/>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-heart-transplantation-assessment/patients/</t>
+          <t>https://www.natera.com/organ-health/prospera-organ-transplantation-assessment/clinicians/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Prospera™ for Kidney Clinician</t>
+          <t>Prospera™ for Kidney Patients</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr"/>
@@ -14779,14 +14747,14 @@
       <c r="E36" s="6" t="inlineStr"/>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-organ-transplantation-assessment/clinicians/</t>
+          <t>https://www.natera.com/organ-health/prospera-organ-transplantation-assessment/patients/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>Prospera™ for Kidney Patients</t>
+          <t>Prospera™ for Lung Patients</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr"/>
@@ -14801,14 +14769,14 @@
       <c r="E37" s="7" t="inlineStr"/>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-organ-transplantation-assessment/patients/</t>
+          <t>https://www.natera.com/organ-health/prospera-lung-transplantation-assessment/patients/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Prospera™ for Lung Patients</t>
+          <t>Renasight™ Clinician Information</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr"/>
@@ -14823,14 +14791,14 @@
       <c r="E38" s="6" t="inlineStr"/>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/prospera-lung-transplantation-assessment/patients/</t>
+          <t>https://www.natera.com/organ-health/renasight-genetic-testing/clinicians/#pg-menu-tabs</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>Renasight™ Clinician Information</t>
+          <t>Renasight™ Gene Conditions List</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr"/>
@@ -14845,14 +14813,14 @@
       <c r="E39" s="7" t="inlineStr"/>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/renasight-genetic-testing/clinicians/#pg-menu-tabs</t>
+          <t>https://www.natera.com/organ-health/renasight-genetic-testing/gene-conditions-list/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Renasight™ Gene Conditions List</t>
+          <t>Renasight™ Patient Information</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr"/>
@@ -14867,14 +14835,14 @@
       <c r="E40" s="6" t="inlineStr"/>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/renasight-genetic-testing/gene-conditions-list/</t>
+          <t>https://www.natera.com/organ-health/renasight-genetic-testing/patients/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>Renasight™ Patient Information</t>
+          <t>Renasight™–Kidney Gene Panel</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr"/>
@@ -14889,14 +14857,14 @@
       <c r="E41" s="7" t="inlineStr"/>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/renasight-genetic-testing/patients/</t>
+          <t>https://www.natera.com/organ-health/renasight-genetic-testing/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Renasight™–Kidney Gene Panel</t>
+          <t>Signatera™ Clinician Information</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr"/>
@@ -14911,14 +14879,14 @@
       <c r="E42" s="6" t="inlineStr"/>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/organ-health/renasight-genetic-testing/</t>
+          <t>https://www.natera.com/oncology/signatera-advanced-cancer-detection/clinicians/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>Signatera™ Clinician Information</t>
+          <t>Signatera™ Patient Information</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr"/>
@@ -14933,14 +14901,14 @@
       <c r="E43" s="7" t="inlineStr"/>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/oncology/signatera-advanced-cancer-detection/clinicians/</t>
+          <t>https://www.natera.com/oncology/signatera-advanced-cancer-detection/patients/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Signatera™ Patient Information</t>
+          <t>Signatera™–Residual Disease Test (MRD)</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr"/>
@@ -14955,14 +14923,14 @@
       <c r="E44" s="6" t="inlineStr"/>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/oncology/signatera-advanced-cancer-detection/patients/</t>
+          <t>https://www.natera.com/oncology/signatera-advanced-cancer-detection/</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>Signatera™–Residual Disease Test (MRD)</t>
+          <t>Vasistera™–Limited Noninvasive Prenatal Testing (NIPT)</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr"/>
@@ -14977,14 +14945,14 @@
       <c r="E45" s="7" t="inlineStr"/>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>https://www.natera.com/oncology/signatera-advanced-cancer-detection/</t>
+          <t>https://www.natera.com/womens-health/vasistera/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Vasistera™–Limited Noninvasive Prenatal Testing (NIPT)</t>
+          <t>Vistara™–Single-Gene NIPT</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr"/>
@@ -14999,20 +14967,20 @@
       <c r="E46" s="6" t="inlineStr"/>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>https://www.natera.com/womens-health/vasistera/</t>
+          <t>https://www.natera.com/womens-health/vistara-nipt-single-gene-test/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>Vistara™–Single-Gene NIPT</t>
+          <t>Women’s Health</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr"/>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Womens Health</t>
+          <t>Organ Health</t>
         </is>
       </c>
       <c r="D47" s="4" t="n">
@@ -15020,28 +14988,6 @@
       </c>
       <c r="E47" s="7" t="inlineStr"/>
       <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>https://www.natera.com/womens-health/vistara-nipt-single-gene-test/</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>Women’s Health</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="inlineStr"/>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>Organ Health</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" s="6" t="inlineStr"/>
-      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>https://www.natera.com/womens-health/</t>
         </is>

</xml_diff>

<commit_message>
chore: scrape results 2026-10-26
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -511,7 +511,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Genetic Panel Scraper — Summary  |  2026-10-19</t>
+          <t>Genetic Panel Scraper — Summary  |  2026-10-26</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       <c r="D6" s="5" t="inlineStr"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -977,7 +977,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1005,7 +1005,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1257,7 +1257,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1397,7 +1397,7 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1569,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1877,7 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2073,7 @@
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2213,7 +2213,7 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2493,7 +2493,7 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2549,7 +2549,7 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2605,7 +2605,7 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2633,7 @@
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2717,7 +2717,7 @@
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="H79" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="H83" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="H85" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3117,7 +3117,7 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="H89" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3173,7 +3173,7 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="H91" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="H93" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3289,7 +3289,7 @@
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="H95" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3373,7 +3373,7 @@
       </c>
       <c r="H97" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="H99" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3461,7 +3461,7 @@
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="H101" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="H103" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3573,7 +3573,7 @@
       </c>
       <c r="H104" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="H105" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3633,7 +3633,7 @@
       </c>
       <c r="H106" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="H107" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3689,7 +3689,7 @@
       </c>
       <c r="H108" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="H109" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3745,7 @@
       </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3777,7 +3777,7 @@
       </c>
       <c r="H111" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3805,7 +3805,7 @@
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="H113" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3889,7 +3889,7 @@
       </c>
       <c r="H115" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3917,7 +3917,7 @@
       </c>
       <c r="H116" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3945,7 +3945,7 @@
       </c>
       <c r="H117" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="H119" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4029,7 +4029,7 @@
       </c>
       <c r="H120" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="H121" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="H122" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4113,7 +4113,7 @@
       </c>
       <c r="H123" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4141,7 @@
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4169,7 +4169,7 @@
       </c>
       <c r="H125" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="H126" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4225,7 +4225,7 @@
       </c>
       <c r="H127" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4253,7 +4253,7 @@
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="H129" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4309,7 +4309,7 @@
       </c>
       <c r="H130" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4337,7 +4337,7 @@
       </c>
       <c r="H131" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4365,7 +4365,7 @@
       </c>
       <c r="H132" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4393,7 +4393,7 @@
       </c>
       <c r="H133" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4421,7 +4421,7 @@
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4449,7 +4449,7 @@
       </c>
       <c r="H135" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4477,7 +4477,7 @@
       </c>
       <c r="H136" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="H137" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4533,7 +4533,7 @@
       </c>
       <c r="H138" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4561,7 @@
       </c>
       <c r="H139" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4589,7 +4589,7 @@
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4617,7 +4617,7 @@
       </c>
       <c r="H141" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4645,7 +4645,7 @@
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="H143" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4705,7 +4705,7 @@
       </c>
       <c r="H144" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4733,7 +4733,7 @@
       </c>
       <c r="H145" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4761,7 +4761,7 @@
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4789,7 +4789,7 @@
       </c>
       <c r="H147" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4817,7 +4817,7 @@
       </c>
       <c r="H148" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="H149" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4873,7 +4873,7 @@
       </c>
       <c r="H150" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="H151" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4929,7 +4929,7 @@
       </c>
       <c r="H152" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="H153" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4985,7 +4985,7 @@
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5013,7 +5013,7 @@
       </c>
       <c r="H155" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5041,7 +5041,7 @@
       </c>
       <c r="H156" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5069,7 +5069,7 @@
       </c>
       <c r="H157" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5097,7 +5097,7 @@
       </c>
       <c r="H158" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5125,7 +5125,7 @@
       </c>
       <c r="H159" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="H160" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5181,7 +5181,7 @@
       </c>
       <c r="H161" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5213,7 +5213,7 @@
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5241,7 +5241,7 @@
       </c>
       <c r="H163" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5269,7 +5269,7 @@
       </c>
       <c r="H164" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5297,7 +5297,7 @@
       </c>
       <c r="H165" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5329,7 +5329,7 @@
       </c>
       <c r="H166" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5357,7 +5357,7 @@
       </c>
       <c r="H167" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5413,7 +5413,7 @@
       </c>
       <c r="H169" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5441,7 +5441,7 @@
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="H171" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5497,7 +5497,7 @@
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5525,7 +5525,7 @@
       </c>
       <c r="H173" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="H174" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5581,7 +5581,7 @@
       </c>
       <c r="H175" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5613,7 +5613,7 @@
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5641,7 +5641,7 @@
       </c>
       <c r="H177" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5673,7 +5673,7 @@
       </c>
       <c r="H178" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5701,7 @@
       </c>
       <c r="H179" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5729,7 +5729,7 @@
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5757,7 +5757,7 @@
       </c>
       <c r="H181" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5785,7 +5785,7 @@
       </c>
       <c r="H182" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5813,7 +5813,7 @@
       </c>
       <c r="H183" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5845,7 +5845,7 @@
       </c>
       <c r="H184" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5873,7 +5873,7 @@
       </c>
       <c r="H185" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5901,7 +5901,7 @@
       </c>
       <c r="H186" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5929,7 +5929,7 @@
       </c>
       <c r="H187" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5957,7 +5957,7 @@
       </c>
       <c r="H188" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5989,7 +5989,7 @@
       </c>
       <c r="H189" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6017,7 +6017,7 @@
       </c>
       <c r="H190" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6045,7 +6045,7 @@
       </c>
       <c r="H191" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6073,7 +6073,7 @@
       </c>
       <c r="H192" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6101,7 +6101,7 @@
       </c>
       <c r="H193" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6129,7 +6129,7 @@
       </c>
       <c r="H194" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6157,7 +6157,7 @@
       </c>
       <c r="H195" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6189,7 +6189,7 @@
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6217,7 +6217,7 @@
       </c>
       <c r="H197" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6245,7 +6245,7 @@
       </c>
       <c r="H198" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6273,7 +6273,7 @@
       </c>
       <c r="H199" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6301,7 +6301,7 @@
       </c>
       <c r="H200" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="H201" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6357,7 @@
       </c>
       <c r="H202" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6385,7 +6385,7 @@
       </c>
       <c r="H203" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6413,7 +6413,7 @@
       </c>
       <c r="H204" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
       </c>
       <c r="H205" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6473,7 +6473,7 @@
       </c>
       <c r="H206" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6501,7 +6501,7 @@
       </c>
       <c r="H207" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6529,7 +6529,7 @@
       </c>
       <c r="H208" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6557,7 +6557,7 @@
       </c>
       <c r="H209" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6585,7 +6585,7 @@
       </c>
       <c r="H210" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6613,7 +6613,7 @@
       </c>
       <c r="H211" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6641,7 +6641,7 @@
       </c>
       <c r="H212" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6669,7 +6669,7 @@
       </c>
       <c r="H213" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6697,7 +6697,7 @@
       </c>
       <c r="H214" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6725,7 +6725,7 @@
       </c>
       <c r="H215" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6753,7 +6753,7 @@
       </c>
       <c r="H216" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6781,7 +6781,7 @@
       </c>
       <c r="H217" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6809,7 +6809,7 @@
       </c>
       <c r="H218" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6837,7 +6837,7 @@
       </c>
       <c r="H219" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6865,7 +6865,7 @@
       </c>
       <c r="H220" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6893,7 +6893,7 @@
       </c>
       <c r="H221" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="H222" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6949,7 +6949,7 @@
       </c>
       <c r="H223" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="H224" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7009,7 +7009,7 @@
       </c>
       <c r="H225" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7037,7 +7037,7 @@
       </c>
       <c r="H226" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="H227" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7093,7 +7093,7 @@
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7121,7 +7121,7 @@
       </c>
       <c r="H229" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="H230" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7177,7 +7177,7 @@
       </c>
       <c r="H231" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7205,7 +7205,7 @@
       </c>
       <c r="H232" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7233,7 +7233,7 @@
       </c>
       <c r="H233" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7261,7 +7261,7 @@
       </c>
       <c r="H234" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7289,7 +7289,7 @@
       </c>
       <c r="H235" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7317,7 +7317,7 @@
       </c>
       <c r="H236" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7345,7 +7345,7 @@
       </c>
       <c r="H237" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7373,7 +7373,7 @@
       </c>
       <c r="H238" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7401,7 +7401,7 @@
       </c>
       <c r="H239" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7429,7 +7429,7 @@
       </c>
       <c r="H240" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7457,7 +7457,7 @@
       </c>
       <c r="H241" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7485,7 +7485,7 @@
       </c>
       <c r="H242" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7513,7 +7513,7 @@
       </c>
       <c r="H243" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7541,7 +7541,7 @@
       </c>
       <c r="H244" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7569,7 +7569,7 @@
       </c>
       <c r="H245" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7597,7 +7597,7 @@
       </c>
       <c r="H246" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7625,7 +7625,7 @@
       </c>
       <c r="H247" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7653,7 +7653,7 @@
       </c>
       <c r="H248" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7681,7 +7681,7 @@
       </c>
       <c r="H249" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7709,7 +7709,7 @@
       </c>
       <c r="H250" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7737,7 +7737,7 @@
       </c>
       <c r="H251" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7765,7 +7765,7 @@
       </c>
       <c r="H252" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7793,7 +7793,7 @@
       </c>
       <c r="H253" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7825,7 +7825,7 @@
       </c>
       <c r="H254" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7857,7 +7857,7 @@
       </c>
       <c r="H255" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7889,7 +7889,7 @@
       </c>
       <c r="H256" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7921,7 +7921,7 @@
       </c>
       <c r="H257" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7953,7 +7953,7 @@
       </c>
       <c r="H258" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -7985,7 +7985,7 @@
       </c>
       <c r="H259" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8017,7 +8017,7 @@
       </c>
       <c r="H260" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8049,7 +8049,7 @@
       </c>
       <c r="H261" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="H262" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8113,7 +8113,7 @@
       </c>
       <c r="H263" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8145,7 +8145,7 @@
       </c>
       <c r="H264" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8177,7 +8177,7 @@
       </c>
       <c r="H265" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8209,7 +8209,7 @@
       </c>
       <c r="H266" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8241,7 +8241,7 @@
       </c>
       <c r="H267" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8273,7 +8273,7 @@
       </c>
       <c r="H268" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8305,7 +8305,7 @@
       </c>
       <c r="H269" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8337,7 +8337,7 @@
       </c>
       <c r="H270" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8369,7 +8369,7 @@
       </c>
       <c r="H271" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8401,7 +8401,7 @@
       </c>
       <c r="H272" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8433,7 +8433,7 @@
       </c>
       <c r="H273" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8465,7 +8465,7 @@
       </c>
       <c r="H274" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8497,7 +8497,7 @@
       </c>
       <c r="H275" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8529,7 +8529,7 @@
       </c>
       <c r="H276" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8561,7 +8561,7 @@
       </c>
       <c r="H277" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8593,7 +8593,7 @@
       </c>
       <c r="H278" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8625,7 +8625,7 @@
       </c>
       <c r="H279" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8657,7 +8657,7 @@
       </c>
       <c r="H280" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8689,7 +8689,7 @@
       </c>
       <c r="H281" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8721,7 +8721,7 @@
       </c>
       <c r="H282" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8753,7 +8753,7 @@
       </c>
       <c r="H283" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8785,7 +8785,7 @@
       </c>
       <c r="H284" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8817,7 +8817,7 @@
       </c>
       <c r="H285" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8849,7 +8849,7 @@
       </c>
       <c r="H286" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8881,7 +8881,7 @@
       </c>
       <c r="H287" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8913,7 +8913,7 @@
       </c>
       <c r="H288" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8945,7 +8945,7 @@
       </c>
       <c r="H289" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -8977,7 +8977,7 @@
       </c>
       <c r="H290" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -9009,7 +9009,7 @@
       </c>
       <c r="H291" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -9041,7 +9041,7 @@
       </c>
       <c r="H292" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -9073,7 +9073,7 @@
       </c>
       <c r="H293" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -9105,7 +9105,7 @@
       </c>
       <c r="H294" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -9137,7 +9137,7 @@
       </c>
       <c r="H295" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -9169,7 +9169,7 @@
       </c>
       <c r="H296" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -9201,7 +9201,7 @@
       </c>
       <c r="H297" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -9233,7 +9233,7 @@
       </c>
       <c r="H298" s="3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -9265,7 +9265,7 @@
       </c>
       <c r="H299" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>

</xml_diff>